<commit_message>
chore(secretos): deprecar URIs de sismo-v3 tras migracion
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/INVENTARIO-SECRETOS.xlsx
+++ b/docs/INVENTARIO-SECRETOS.xlsx
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Render env (compas-api)</t>
+          <t>Render env (compas-api) | DEPRECADA 2026-09-15 - migrado a compas-prod</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Render env (compas-api)</t>
+          <t>Render env (compas-api) | DEPRECADA 2026-09-15 - migrado a compas-prod</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">

</xml_diff>